<commit_message>
push on october 2026
</commit_message>
<xml_diff>
--- a/sales_app/data/Full Plan workflow.xlsx
+++ b/sales_app/data/Full Plan workflow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macintoshi/Desktop/Django_unchainded/sales_app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF7C06D8-5BE5-D542-8105-1C869EE4F491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23A61C05-D9D4-B046-87CB-8052FF646735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="22020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1270" uniqueCount="94">
   <si>
     <t>location</t>
   </si>
@@ -548,6 +548,9 @@
   <si>
     <t>ჯამი</t>
   </si>
+  <si>
+    <t>გუდვილი 2</t>
+  </si>
 </sst>
 </file>
 
@@ -821,7 +824,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -887,6 +890,8 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6746,7 +6751,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{650603AD-9288-4A14-8188-833FDDD6C46C}">
-  <dimension ref="A1:K463"/>
+  <dimension ref="A1:K475"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="7" width="21.1640625" style="24"/>
@@ -16826,6 +16831,210 @@
       </c>
       <c r="E463">
         <v>63000</v>
+      </c>
+    </row>
+    <row r="464" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A464">
+        <v>2026</v>
+      </c>
+      <c r="B464">
+        <v>10</v>
+      </c>
+      <c r="C464" t="s">
+        <v>1</v>
+      </c>
+      <c r="D464" t="s">
+        <v>62</v>
+      </c>
+      <c r="E464">
+        <v>123000</v>
+      </c>
+    </row>
+    <row r="465" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A465">
+        <v>2026</v>
+      </c>
+      <c r="B465">
+        <v>10</v>
+      </c>
+      <c r="C465" t="s">
+        <v>2</v>
+      </c>
+      <c r="D465" t="s">
+        <v>55</v>
+      </c>
+      <c r="E465">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="466" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A466">
+        <v>2026</v>
+      </c>
+      <c r="B466">
+        <v>10</v>
+      </c>
+      <c r="C466" t="s">
+        <v>3</v>
+      </c>
+      <c r="D466" t="s">
+        <v>48</v>
+      </c>
+      <c r="E466">
+        <v>59000</v>
+      </c>
+    </row>
+    <row r="467" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A467">
+        <v>2026</v>
+      </c>
+      <c r="B467">
+        <v>10</v>
+      </c>
+      <c r="C467" t="s">
+        <v>4</v>
+      </c>
+      <c r="D467" t="s">
+        <v>63</v>
+      </c>
+      <c r="E467">
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="468" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A468">
+        <v>2026</v>
+      </c>
+      <c r="B468">
+        <v>10</v>
+      </c>
+      <c r="C468" t="s">
+        <v>5</v>
+      </c>
+      <c r="D468" t="s">
+        <v>54</v>
+      </c>
+      <c r="E468">
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="469" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A469">
+        <v>2026</v>
+      </c>
+      <c r="B469">
+        <v>10</v>
+      </c>
+      <c r="C469" t="s">
+        <v>6</v>
+      </c>
+      <c r="D469" t="s">
+        <v>57</v>
+      </c>
+      <c r="E469">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="470" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A470">
+        <v>2026</v>
+      </c>
+      <c r="B470">
+        <v>10</v>
+      </c>
+      <c r="C470" t="s">
+        <v>7</v>
+      </c>
+      <c r="D470" t="s">
+        <v>64</v>
+      </c>
+      <c r="E470">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="471" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A471">
+        <v>2026</v>
+      </c>
+      <c r="B471">
+        <v>10</v>
+      </c>
+      <c r="C471" t="s">
+        <v>8</v>
+      </c>
+      <c r="D471" t="s">
+        <v>58</v>
+      </c>
+      <c r="E471">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="472" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A472">
+        <v>2026</v>
+      </c>
+      <c r="B472">
+        <v>10</v>
+      </c>
+      <c r="C472" t="s">
+        <v>9</v>
+      </c>
+      <c r="D472" t="s">
+        <v>49</v>
+      </c>
+      <c r="E472">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="473" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A473">
+        <v>2026</v>
+      </c>
+      <c r="B473">
+        <v>10</v>
+      </c>
+      <c r="C473" t="s">
+        <v>10</v>
+      </c>
+      <c r="D473" t="s">
+        <v>50</v>
+      </c>
+      <c r="E473">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="474" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A474">
+        <v>2026</v>
+      </c>
+      <c r="B474">
+        <v>10</v>
+      </c>
+      <c r="C474" t="s">
+        <v>11</v>
+      </c>
+      <c r="D474" t="s">
+        <v>59</v>
+      </c>
+      <c r="E474">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="475" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A475">
+        <v>2026</v>
+      </c>
+      <c r="B475">
+        <v>10</v>
+      </c>
+      <c r="C475" t="s">
+        <v>12</v>
+      </c>
+      <c r="D475" t="s">
+        <v>60</v>
+      </c>
+      <c r="E475">
+        <v>59000</v>
       </c>
     </row>
   </sheetData>
@@ -17082,12 +17291,13 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51FCE611-90D9-BD45-9A96-E3469C310DDF}">
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.83203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -17585,7 +17795,7 @@
         <v>705000</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
         <v>65</v>
       </c>
@@ -17599,7 +17809,7 @@
         <v>121000</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
         <v>66</v>
       </c>
@@ -17612,8 +17822,26 @@
       <c r="D18">
         <v>87000</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G18" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="H18" s="33">
+        <v>59000</v>
+      </c>
+      <c r="I18" s="33">
+        <v>50150</v>
+      </c>
+      <c r="L18" s="48" t="s">
+        <v>1</v>
+      </c>
+      <c r="M18" s="48" t="s">
+        <v>62</v>
+      </c>
+      <c r="N18">
+        <v>123000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
         <v>67</v>
       </c>
@@ -17626,8 +17854,26 @@
       <c r="D19">
         <v>57000</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G19" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="H19" s="33">
+        <v>57000</v>
+      </c>
+      <c r="I19" s="33">
+        <v>48450</v>
+      </c>
+      <c r="L19" s="47" t="s">
+        <v>2</v>
+      </c>
+      <c r="M19" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="N19">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
         <v>68</v>
       </c>
@@ -17640,8 +17886,26 @@
       <c r="D20">
         <v>55000</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G20" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="H20" s="33">
+        <v>123000</v>
+      </c>
+      <c r="I20" s="33">
+        <v>104550</v>
+      </c>
+      <c r="L20" s="48" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="N20">
+        <v>59000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
         <v>69</v>
       </c>
@@ -17654,8 +17918,26 @@
       <c r="D21">
         <v>67000</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G21" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="H21" s="33">
+        <v>45000</v>
+      </c>
+      <c r="I21" s="33">
+        <v>38250</v>
+      </c>
+      <c r="L21" s="47" t="s">
+        <v>4</v>
+      </c>
+      <c r="M21" s="47" t="s">
+        <v>63</v>
+      </c>
+      <c r="N21">
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
         <v>70</v>
       </c>
@@ -17668,8 +17950,26 @@
       <c r="D22">
         <v>44000</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G22" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="H22" s="33">
+        <v>40000</v>
+      </c>
+      <c r="I22" s="33">
+        <v>34000</v>
+      </c>
+      <c r="L22" s="48" t="s">
+        <v>5</v>
+      </c>
+      <c r="M22" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="N22">
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="33" t="s">
         <v>71</v>
       </c>
@@ -17682,8 +17982,26 @@
       <c r="D23">
         <v>42000</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G23" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="H23" s="33">
+        <v>85000</v>
+      </c>
+      <c r="I23" s="33">
+        <v>72250</v>
+      </c>
+      <c r="L23" s="47" t="s">
+        <v>6</v>
+      </c>
+      <c r="M23" s="47" t="s">
+        <v>57</v>
+      </c>
+      <c r="N23">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="33" t="s">
         <v>72</v>
       </c>
@@ -17696,8 +18014,26 @@
       <c r="D24">
         <v>48000</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G24" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="H24" s="33">
+        <v>42000</v>
+      </c>
+      <c r="I24" s="33">
+        <v>35700</v>
+      </c>
+      <c r="L24" s="48" t="s">
+        <v>7</v>
+      </c>
+      <c r="M24" s="48" t="s">
+        <v>64</v>
+      </c>
+      <c r="N24">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="33" t="s">
         <v>73</v>
       </c>
@@ -17710,8 +18046,26 @@
       <c r="D25">
         <v>30000</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G25" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="H25" s="33">
+        <v>48000</v>
+      </c>
+      <c r="I25" s="33">
+        <v>40800</v>
+      </c>
+      <c r="L25" s="47" t="s">
+        <v>8</v>
+      </c>
+      <c r="M25" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="N25">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="33" t="s">
         <v>74</v>
       </c>
@@ -17724,8 +18078,26 @@
       <c r="D26">
         <v>45000</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G26" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="H26" s="33">
+        <v>45000</v>
+      </c>
+      <c r="I26" s="33">
+        <v>38250</v>
+      </c>
+      <c r="L26" s="48" t="s">
+        <v>9</v>
+      </c>
+      <c r="M26" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="N26">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="33" t="s">
         <v>75</v>
       </c>
@@ -17738,8 +18110,26 @@
       <c r="D27">
         <v>46000</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G27" s="33" t="s">
+        <v>49</v>
+      </c>
+      <c r="H27" s="33">
+        <v>30000</v>
+      </c>
+      <c r="I27" s="33">
+        <v>25500</v>
+      </c>
+      <c r="L27" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="M27" s="47" t="s">
+        <v>50</v>
+      </c>
+      <c r="N27">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="33" t="s">
         <v>76</v>
       </c>
@@ -17752,8 +18142,26 @@
       <c r="D28">
         <v>63000</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G28" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="H28" s="33">
+        <v>59000</v>
+      </c>
+      <c r="I28" s="33">
+        <v>50150</v>
+      </c>
+      <c r="L28" s="48" t="s">
+        <v>11</v>
+      </c>
+      <c r="M28" s="48" t="s">
+        <v>59</v>
+      </c>
+      <c r="N28">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="33" t="s">
         <v>77</v>
       </c>
@@ -17762,6 +18170,33 @@
       </c>
       <c r="C29" s="33">
         <v>13600</v>
+      </c>
+      <c r="G29" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="H29" s="33">
+        <v>57000</v>
+      </c>
+      <c r="I29" s="33">
+        <v>48450</v>
+      </c>
+      <c r="L29" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="M29" s="47" t="s">
+        <v>60</v>
+      </c>
+      <c r="N29">
+        <v>59000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="G30" s="33"/>
+      <c r="H30" s="33">
+        <v>690000</v>
+      </c>
+      <c r="I30" s="33">
+        <v>586500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>